<commit_message>
final changes to FIM 4.30/5.5
</commit_message>
<xml_diff>
--- a/results/05-2026/beta/contributions-05-2026.xlsx
+++ b/results/05-2026/beta/contributions-05-2026.xlsx
@@ -3036,7 +3036,7 @@
         <v>-0.0000531438557844164</v>
       </c>
       <c r="W25" t="n">
-        <v>0.338301811894314</v>
+        <v>0.283001238493291</v>
       </c>
       <c r="X25" t="n">
         <v>0.0427711776553399</v>
@@ -3051,22 +3051,22 @@
         <v>-0.270169588737866</v>
       </c>
       <c r="AB25" t="n">
-        <v>0.408480143900867</v>
+        <v>0.353220653663715</v>
       </c>
       <c r="AC25" t="n">
-        <v>0.139473515989945</v>
+        <v>0.0840566015320863</v>
       </c>
       <c r="AD25" t="n">
         <v>-0.412652726526158</v>
       </c>
       <c r="AE25" t="n">
-        <v>0.432744756378526</v>
+        <v>0.377485266141373</v>
       </c>
       <c r="AF25" t="n">
-        <v>-1.17826914678364</v>
+        <v>-1.2336860612415</v>
       </c>
       <c r="AG25" t="n">
-        <v>-0.49086414168114</v>
+        <v>-0.504718370295605</v>
       </c>
     </row>
     <row r="26">
@@ -3137,7 +3137,7 @@
         <v>-0.0000696617484409661</v>
       </c>
       <c r="W26" t="n">
-        <v>0.279329039690738</v>
+        <v>0.224985702190415</v>
       </c>
       <c r="X26" t="n">
         <v>0.0124692193307716</v>
@@ -3152,22 +3152,22 @@
         <v>0.463404670727734</v>
       </c>
       <c r="AB26" t="n">
-        <v>-0.00467134528318946</v>
+        <v>-0.059175626483968</v>
       </c>
       <c r="AC26" t="n">
-        <v>0.518755843342824</v>
+        <v>0.464514269397324</v>
       </c>
       <c r="AD26" t="n">
         <v>0.148888893636348</v>
       </c>
       <c r="AE26" t="n">
-        <v>-0.00341842784719892</v>
+        <v>-0.0579227090479775</v>
       </c>
       <c r="AF26" t="n">
-        <v>0.884206322384365</v>
+        <v>0.829964748438865</v>
       </c>
       <c r="AG26" t="n">
-        <v>-0.103496105815382</v>
+        <v>-0.130910727916221</v>
       </c>
     </row>
     <row r="27">
@@ -3238,10 +3238,10 @@
         <v>-0.000501429966115183</v>
       </c>
       <c r="W27" t="n">
-        <v>0.247504863679855</v>
+        <v>0.207022102238222</v>
       </c>
       <c r="X27" t="n">
-        <v>0.0487650643212487</v>
+        <v>0.0365288260044681</v>
       </c>
       <c r="Y27" t="n">
         <v>-0.330545226387455</v>
@@ -3253,22 +3253,22 @@
         <v>0.485607963229528</v>
       </c>
       <c r="AB27" t="n">
-        <v>0.0416926751894501</v>
+        <v>-0.0111200504906592</v>
       </c>
       <c r="AC27" t="n">
-        <v>0.587088193681598</v>
+        <v>0.534544569658873</v>
       </c>
       <c r="AD27" t="n">
         <v>0.234064323299038</v>
       </c>
       <c r="AE27" t="n">
-        <v>0.0447763327104476</v>
+        <v>-0.00803639296966173</v>
       </c>
       <c r="AF27" t="n">
-        <v>0.163659314276233</v>
+        <v>0.111115690253508</v>
       </c>
       <c r="AG27" t="n">
-        <v>0.0398941382049361</v>
+        <v>-0.000656389901584911</v>
       </c>
     </row>
     <row r="28">
@@ -3282,7 +3282,7 @@
         <v>0</v>
       </c>
       <c r="D28" t="n">
-        <v>-0.146342913256379</v>
+        <v>-0.30586383600656</v>
       </c>
       <c r="E28" t="n">
         <v>-0.176236422781678</v>
@@ -3339,13 +3339,13 @@
         <v>-0.000426940925803921</v>
       </c>
       <c r="W28" t="n">
-        <v>0.200762093320125</v>
+        <v>0.162770134174828</v>
       </c>
       <c r="X28" t="n">
-        <v>-0.0141682460370789</v>
+        <v>-0.0273950236581683</v>
       </c>
       <c r="Y28" t="n">
-        <v>-0.182706291067979</v>
+        <v>-0.34222721381816</v>
       </c>
       <c r="Z28" t="n">
         <v>-0.139873044970078</v>
@@ -3354,22 +3354,22 @@
         <v>0.255014185511323</v>
       </c>
       <c r="AB28" t="n">
-        <v>0.128159277609808</v>
+        <v>0.0769259524623977</v>
       </c>
       <c r="AC28" t="n">
-        <v>0.442829230353156</v>
+        <v>0.391733535269023</v>
       </c>
       <c r="AD28" t="n">
         <v>0.177083575542115</v>
       </c>
       <c r="AE28" t="n">
-        <v>0.123898637736446</v>
+        <v>0.0726653125890352</v>
       </c>
       <c r="AF28" t="n">
-        <v>0.120249894315099</v>
+        <v>-0.0903667235192149</v>
       </c>
       <c r="AG28" t="n">
-        <v>-0.00253840395198553</v>
+        <v>-0.095743086517085</v>
       </c>
     </row>
     <row r="29">
@@ -3383,7 +3383,7 @@
         <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>-0.10687586310228</v>
+        <v>-0.106184459909413</v>
       </c>
       <c r="E29" t="n">
         <v>-0.199946813675512</v>
@@ -3440,13 +3440,13 @@
         <v>-0.000395175505607586</v>
       </c>
       <c r="W29" t="n">
-        <v>0.164055586793484</v>
+        <v>0.110104285704918</v>
       </c>
       <c r="X29" t="n">
-        <v>0.0153627081459999</v>
+        <v>-0.0142421131305181</v>
       </c>
       <c r="Y29" t="n">
-        <v>-0.165982905043573</v>
+        <v>-0.165291501850706</v>
       </c>
       <c r="Z29" t="n">
         <v>-0.140839771734219</v>
@@ -3455,22 +3455,22 @@
         <v>-0.0600454191026175</v>
       </c>
       <c r="AB29" t="n">
-        <v>0.17980531124795</v>
+        <v>0.0962927443821378</v>
       </c>
       <c r="AC29" t="n">
-        <v>0.179873938990407</v>
+        <v>0.096308392813431</v>
       </c>
       <c r="AD29" t="n">
         <v>-0.00775380490190472</v>
       </c>
       <c r="AE29" t="n">
-        <v>0.171173759027019</v>
+        <v>0.0876611921612072</v>
       </c>
       <c r="AF29" t="n">
-        <v>-0.126948737787385</v>
+        <v>-0.209822880771494</v>
       </c>
       <c r="AG29" t="n">
-        <v>0.260291698297078</v>
+        <v>0.160222708600416</v>
       </c>
     </row>
     <row r="30">
@@ -3484,7 +3484,7 @@
         <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.11397551834177</v>
+        <v>-0.113238185935717</v>
       </c>
       <c r="E30" t="n">
         <v>-0.186214773942108</v>
@@ -3541,13 +3541,13 @@
         <v>-0.000365697253103981</v>
       </c>
       <c r="W30" t="n">
-        <v>0.125233288715792</v>
+        <v>0.0747419360682316</v>
       </c>
       <c r="X30" t="n">
-        <v>0.0224941043379145</v>
+        <v>-0.00432257924151644</v>
       </c>
       <c r="Y30" t="n">
-        <v>-0.1602387861888</v>
+        <v>-0.159501453782747</v>
       </c>
       <c r="Z30" t="n">
         <v>-0.139951506095078</v>
@@ -3556,22 +3556,22 @@
         <v>-0.533901846857373</v>
       </c>
       <c r="AB30" t="n">
-        <v>0.264760058414852</v>
+        <v>0.18758138864818</v>
       </c>
       <c r="AC30" t="n">
-        <v>-0.207644369916542</v>
+        <v>-0.285259688698547</v>
       </c>
       <c r="AD30" t="n">
         <v>-0.267027899335481</v>
       </c>
       <c r="AE30" t="n">
-        <v>0.262385836880811</v>
+        <v>0.18520716711414</v>
       </c>
       <c r="AF30" t="n">
-        <v>-0.50783466220042</v>
+        <v>-0.584712648576373</v>
       </c>
       <c r="AG30" t="n">
-        <v>-0.0877185478491185</v>
+        <v>-0.193446640653394</v>
       </c>
     </row>
     <row r="31">
@@ -3585,7 +3585,7 @@
         <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.0975287813488231</v>
+        <v>-0.0968978464598438</v>
       </c>
       <c r="E31" t="n">
         <v>-0.18074145350152</v>
@@ -3642,13 +3642,13 @@
         <v>-0.000318458448563437</v>
       </c>
       <c r="W31" t="n">
-        <v>0.119159394811257</v>
+        <v>0.0602243053891414</v>
       </c>
       <c r="X31" t="n">
-        <v>-0.00107466719411561</v>
+        <v>-0.0135877228904138</v>
       </c>
       <c r="Y31" t="n">
-        <v>-0.14208312752099</v>
+        <v>-0.14145219263201</v>
       </c>
       <c r="Z31" t="n">
         <v>-0.136187107329353</v>
@@ -3657,22 +3657,22 @@
         <v>-0.484036400696089</v>
       </c>
       <c r="AB31" t="n">
-        <v>0.142418793573071</v>
+        <v>0.0709964759778335</v>
       </c>
       <c r="AC31" t="n">
-        <v>-0.280885780310953</v>
+        <v>-0.352675151673145</v>
       </c>
       <c r="AD31" t="n">
         <v>-0.120213984396549</v>
       </c>
       <c r="AE31" t="n">
-        <v>0.142742647755256</v>
+        <v>0.0713203301600185</v>
       </c>
       <c r="AF31" t="n">
-        <v>-0.559156015161296</v>
+        <v>-0.630314451634508</v>
       </c>
       <c r="AG31" t="n">
-        <v>-0.268422380208501</v>
+        <v>-0.378804176125398</v>
       </c>
     </row>
     <row r="32">
@@ -3686,7 +3686,7 @@
         <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.104154696248239</v>
+        <v>-0.103480896875323</v>
       </c>
       <c r="E32" t="n">
         <v>-0.188023408655981</v>
@@ -3743,13 +3743,13 @@
         <v>-0.000312156590467466</v>
       </c>
       <c r="W32" t="n">
-        <v>0.0652367227493609</v>
+        <v>0.0092716635034082</v>
       </c>
       <c r="X32" t="n">
-        <v>-0.0134946507383032</v>
+        <v>-0.0234751031805249</v>
       </c>
       <c r="Y32" t="n">
-        <v>-0.147016752572777</v>
+        <v>-0.146342953199862</v>
       </c>
       <c r="Z32" t="n">
         <v>-0.145161352331443</v>
@@ -3758,22 +3758,22 @@
         <v>-0.260600449467441</v>
       </c>
       <c r="AB32" t="n">
-        <v>0.0804088679384772</v>
+        <v>0.0144763954096759</v>
       </c>
       <c r="AC32" t="n">
-        <v>-0.179969244932549</v>
+        <v>-0.246084030405244</v>
       </c>
       <c r="AD32" t="n">
         <v>0.125828825912292</v>
       </c>
       <c r="AE32" t="n">
-        <v>0.0753714824875317</v>
+        <v>0.00943900995873045</v>
       </c>
       <c r="AF32" t="n">
-        <v>-0.472147349836769</v>
+        <v>-0.537588335936549</v>
       </c>
       <c r="AG32" t="n">
-        <v>-0.416521691246468</v>
+        <v>-0.490609579229731</v>
       </c>
     </row>
     <row r="33">
@@ -3787,7 +3787,7 @@
         <v>0</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.171995982760397</v>
+        <v>-0.170883303356563</v>
       </c>
       <c r="E33" t="n">
         <v>-0.184495417794735</v>
@@ -3844,13 +3844,13 @@
         <v>-0.000305491844496977</v>
       </c>
       <c r="W33" t="n">
-        <v>0.0239552259170439</v>
+        <v>-0.00136295384642158</v>
       </c>
       <c r="X33" t="n">
-        <v>-0.00000458810015208636</v>
+        <v>-0.0115869753952157</v>
       </c>
       <c r="Y33" t="n">
-        <v>-0.213430042513555</v>
+        <v>-0.212317363109721</v>
       </c>
       <c r="Z33" t="n">
         <v>-0.143061358041577</v>
@@ -3859,22 +3859,22 @@
         <v>-0.247370645122349</v>
       </c>
       <c r="AB33" t="n">
-        <v>0.02383117359416</v>
+        <v>-0.0130696093021457</v>
       </c>
       <c r="AC33" t="n">
-        <v>-0.223476852791337</v>
+        <v>-0.260474593853452</v>
       </c>
       <c r="AD33" t="n">
         <v>0.181346316904211</v>
       </c>
       <c r="AE33" t="n">
-        <v>0.0198902270893699</v>
+        <v>-0.0170105558069359</v>
       </c>
       <c r="AF33" t="n">
-        <v>-0.579968253346469</v>
+        <v>-0.615853315004751</v>
       </c>
       <c r="AG33" t="n">
-        <v>-0.529776570136239</v>
+        <v>-0.592117187788045</v>
       </c>
     </row>
     <row r="34">
@@ -3888,7 +3888,7 @@
         <v>0</v>
       </c>
       <c r="D34" t="n">
-        <v>-0.205141427200942</v>
+        <v>-0.203814322711313</v>
       </c>
       <c r="E34" t="n">
         <v>-0.183578043716544</v>
@@ -3945,13 +3945,13 @@
         <v>-0.000299428155345378</v>
       </c>
       <c r="W34" t="n">
-        <v>0.00302249226130404</v>
+        <v>-0.0331773637149976</v>
       </c>
       <c r="X34" t="n">
-        <v>0.0216035681134529</v>
+        <v>0.00776152455226643</v>
       </c>
       <c r="Y34" t="n">
-        <v>-0.245538348742651</v>
+        <v>-0.244211244253022</v>
       </c>
       <c r="Z34" t="n">
         <v>-0.143181122174836</v>
@@ -3960,22 +3960,22 @@
         <v>-0.59681672518361</v>
       </c>
       <c r="AB34" t="n">
-        <v>-0.0527204838840258</v>
+        <v>-0.10280007135667</v>
       </c>
       <c r="AC34" t="n">
-        <v>-0.649871055737251</v>
+        <v>-0.700267708903581</v>
       </c>
       <c r="AD34" t="n">
         <v>0.0200594465950505</v>
       </c>
       <c r="AE34" t="n">
-        <v>-0.0527204838840258</v>
+        <v>-0.10280007135667</v>
       </c>
       <c r="AF34" t="n">
-        <v>-1.03859052665474</v>
+        <v>-1.08766007533144</v>
       </c>
       <c r="AG34" t="n">
-        <v>-0.662465536249818</v>
+        <v>-0.717854044476812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>